<commit_message>
docs: add Venue/Peer-Reviewed column to main Paper Dictionary
13 peer-reviewed, 5 preprints, 2 workshop, 6 unknown (no URL).
Verified via arXiv journal refs and ACL Anthology.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/literature-review/Paper Dictionary.xlsx
+++ b/literature-review/Paper Dictionary.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,8 +35,11 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +62,26 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D6E4F0"/>
         <bgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -108,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -124,6 +147,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -489,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -499,6 +537,7 @@
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -551,6 +590,11 @@
           <t>Open Research Directions</t>
         </is>
       </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>Venue / Peer-Reviewed?</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="40" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -584,6 +628,11 @@
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>✓ NeurIPS 2023</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -617,6 +666,11 @@
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>✗ arXiv preprint (2025) — not peer-reviewed</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -646,6 +700,11 @@
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>Unknown — no URL, verify</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -675,6 +734,11 @@
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>Unknown — no URL, verify</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="40" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -704,6 +768,11 @@
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr"/>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>Unknown — no URL, verify</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -733,6 +802,11 @@
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>Unknown — no URL, verify</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
@@ -766,6 +840,11 @@
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr"/>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>✓ WACV 2025</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -795,6 +874,11 @@
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr"/>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Unknown — no URL, verify</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="40" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
@@ -828,6 +912,11 @@
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>✓ NeurIPS 2020</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -861,6 +950,11 @@
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr"/>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>✗ arXiv preprint (2025) — not peer-reviewed</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="40" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -890,6 +984,11 @@
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr"/>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>Unknown — no URL, verify</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="40" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -923,6 +1022,11 @@
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr"/>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>✓ ICML 2023</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="40" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -956,6 +1060,11 @@
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr"/>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>✓ National Science Review (2024)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="40" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -989,6 +1098,11 @@
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr"/>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>✓ Interspeech 2023</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="40" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
@@ -1022,6 +1136,11 @@
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr"/>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>✓ Interspeech 2024</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="40" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
@@ -1055,6 +1174,11 @@
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr"/>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>Unknown — paywalled, verify</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="40" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
@@ -1088,6 +1212,11 @@
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr"/>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>~ RANLP 2021 Workshop (SRW) (workshop — peer-reviewed)</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="40" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
@@ -1121,6 +1250,11 @@
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr"/>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>✓ MDPI Sensors (2025)</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="40" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
@@ -1150,6 +1284,11 @@
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr"/>
+      <c r="H22" s="10" t="inlineStr">
+        <is>
+          <t>Unknown — no URL, verify</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="40" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
@@ -1183,6 +1322,11 @@
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr"/>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>✓ NeurIPS 2025</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="40" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
@@ -1216,6 +1360,11 @@
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr"/>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>✓ ACL Findings 2025</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="40" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
@@ -1249,6 +1398,11 @@
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr"/>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>✗ arXiv preprint (2025) — not peer-reviewed</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="40" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
@@ -1282,6 +1436,11 @@
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr"/>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>✗ arXiv preprint (2025) — not peer-reviewed</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="40" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
@@ -1315,6 +1474,11 @@
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr"/>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>✓ IEEE Transactions on Multimedia (TMM)</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="40" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
@@ -1348,6 +1512,11 @@
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr"/>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>✓ Springer LNCS conference chapter (peer-reviewed — specific conference, verify)</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="40" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
@@ -1381,6 +1550,11 @@
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr"/>
+      <c r="H29" s="11" t="inlineStr">
+        <is>
+          <t>~ SIGIR 2024 Workshop (MRR) (workshop — peer-reviewed)</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="40" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
@@ -1414,6 +1588,11 @@
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr"/>
+      <c r="H30" s="9" t="inlineStr">
+        <is>
+          <t>✗ arXiv preprint (2026) — not peer-reviewed</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="40" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
@@ -1447,6 +1626,11 @@
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr"/>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t>✗ arXiv preprint (2026) — not peer-reviewed</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="40" customHeight="1">
       <c r="A32" s="3" t="inlineStr">
@@ -1480,6 +1664,11 @@
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr"/>
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>✓ EMNLP 2025</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="40" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
@@ -1513,6 +1702,11 @@
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr"/>
+      <c r="H33" s="8" t="inlineStr">
+        <is>
+          <t>✓ NeurIPS 2025 (Spotlight)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs: add missing URLs and fix venues in main Paper Dictionary
- Add URLs for MovieChat+, VideoABC, Dual-level Dynamic, Temporal
  Grounding Survey, Caption Assisted LLM, RAG Healthcare, CALCE
- Fix all 6 grey 'unknown' venue entries (all are peer-reviewed journals)
- Fix Springer LNCS chapter: AIMSA 2024 conference
- Flag rows 11 and 22 as likely duplicate (Caption Assisted LLM = CALCE)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/literature-review/Paper Dictionary.xlsx
+++ b/literature-review/Paper Dictionary.xlsx
@@ -39,7 +39,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -82,6 +82,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCC99"/>
       </patternFill>
     </fill>
   </fills>
@@ -131,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -160,6 +165,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -678,7 +686,11 @@
           <t>MovieChat+: Question-Aware Sparse Memory for Long Video Question Answering</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2404.17176</t>
+        </is>
+      </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
           <t>MovieChat+ proposes a question-aware sparse memory mechanism for long video QA, selectively compressing video tokens to handle hour-long content without prohibitive memory costs. It demonstrates improved performance over dense-memory baselines on long-video benchmarks.</t>
@@ -700,9 +712,9 @@
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>Unknown — no URL, verify</t>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>✓ IEEE TPAMI 2026 (Transactions on Pattern Analysis and Machine Intelligence)</t>
         </is>
       </c>
     </row>
@@ -712,7 +724,11 @@
           <t>VideoABC: A Real-World Video Dataset for Abductive Visual Reasoning</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr"/>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>https://ieeexplore.ieee.org/document/9893026/</t>
+        </is>
+      </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
           <t>VideoABC introduces abductive visual reasoning over instructional videos, requiring models to infer the most plausible explanation for observations across long-term temporal sequences. It uses real-world instructional content, making it closer to lecture settings than typical entertainment video datasets.</t>
@@ -734,9 +750,9 @@
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr"/>
-      <c r="H7" s="10" t="inlineStr">
-        <is>
-          <t>Unknown — no URL, verify</t>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>✓ IEEE TIP 2022 (Transactions on Image Processing)</t>
         </is>
       </c>
     </row>
@@ -746,7 +762,11 @@
           <t>Dual-level Dynamic Heterogeneous Graph Network for Video Question Answering</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sciencedirect.com/science/article/abs/pii/S0893608025009748</t>
+        </is>
+      </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Proposes a dual-level graph network to model entity and event relationships in video QA, addressing the tendency of VLMs to rely on language shortcuts rather than visual grounding. Introduces richer entity/event annotations to improve multi-modal reasoning.</t>
@@ -768,9 +788,9 @@
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="10" t="inlineStr">
-        <is>
-          <t>Unknown — no URL, verify</t>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>✓ Neural Networks, Elsevier (2025)</t>
         </is>
       </c>
     </row>
@@ -780,7 +800,11 @@
           <t>Temporal Sentence Grounding in Videos: A Survey and Future Directions</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr"/>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2201.08071</t>
+        </is>
+      </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
           <t>A comprehensive survey of temporal sentence grounding in videos (TSGV), also known as natural language video localization and video moment retrieval. Covers foundational datasets, evaluation metrics including temporal IoU, and model architectures from proposal-based to proposal-free methods.</t>
@@ -802,9 +826,9 @@
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr"/>
-      <c r="H9" s="10" t="inlineStr">
-        <is>
-          <t>Unknown — no URL, verify</t>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>✓ IEEE TPAMI 2023 (Transactions on Pattern Analysis and Machine Intelligence)</t>
         </is>
       </c>
     </row>
@@ -852,7 +876,11 @@
           <t>Caption Assisted Multimodal Large Language Model for Video Moment Retrieval</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr"/>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>https://ieeexplore.ieee.org/document/11206011</t>
+        </is>
+      </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
           <t>CALCE proposes a two-stage coarse-to-fine framework for video moment retrieval using frame captions to assist multimodal LLMs. Frame captions bridge the gap between visual and textual modalities, improving temporal localization accuracy.</t>
@@ -874,9 +902,9 @@
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr"/>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>Unknown — no URL, verify</t>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>✓ IEEE TIP 2025 — NOTE: same paper as row 22 (CALCE) — possible duplicate entry</t>
         </is>
       </c>
     </row>
@@ -962,7 +990,11 @@
           <t>Retrieval Augmented Generation for Large Language Models in Healthcare: A Systematic Review</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>https://journals.plos.org/digitalhealth/article?id=10.1371/journal.pdig.0000877</t>
+        </is>
+      </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Surveys RAG applications in healthcare, highlighting common failure modes including hallucination, retrieval errors, and citation inaccuracy. Provides a framework for evaluating RAG reliability in high-stakes domains, with metrics applicable to educational QA evaluation.</t>
@@ -984,9 +1016,9 @@
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr"/>
-      <c r="H14" s="10" t="inlineStr">
-        <is>
-          <t>Unknown — no URL, verify</t>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>✓ PLOS Digital Health (2025)</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1294,11 @@
           <t>Caption Assisted Multimodal LLM from Coarse to Fine (CALCE) for Video Moment Retrieval</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>https://ieeexplore.ieee.org/document/11206011</t>
+        </is>
+      </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
           <t>A two-stage coarse-to-fine retrieval framework where frame captions assist MLLMs in localizing specific video moments. The coarse stage narrows candidate segments; the fine stage reranks using multimodal reasoning.</t>
@@ -1284,9 +1320,9 @@
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr"/>
-      <c r="H22" s="10" t="inlineStr">
-        <is>
-          <t>Unknown — no URL, verify</t>
+      <c r="H22" s="12" t="inlineStr">
+        <is>
+          <t>✓ IEEE TIP 2025 — NOTE: same paper as row 11 (Caption Assisted LLM) — possible duplicate entry</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1550,7 @@
       <c r="G28" s="3" t="inlineStr"/>
       <c r="H28" s="8" t="inlineStr">
         <is>
-          <t>✓ Springer LNCS conference chapter (peer-reviewed — specific conference, verify)</t>
+          <t>✓ AIMSA 2024 (19th Intl. Conf. on AI: Methodology, Systems, and Applications), Springer LNCS</t>
         </is>
       </c>
     </row>

</xml_diff>